<commit_message>
Add legal stopwords for improved word cloud generation
</commit_message>
<xml_diff>
--- a/data/history.xlsx
+++ b/data/history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1747,6 +1747,374 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Mahendra_Bhaskar_Limaye_vs_Union_Of_India_Thr_Secretary_on_20_October_2023.PDF</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:06:36.306876</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "1": "Shyam_Lal_vs_1_The_State_Of_Uttar_Pradesh2_The_Union_on_30_March_1954_1.PDF", "2": "T_Cajee_vs_U_Jormanik_Siem_And_Another_on_20_September_1960_1.PDF", "3": "Kanumukkala_Krishna_Murthy_vs_State_Of_Andhra_Pradesh_on_23_March_1964_1.PDF", "4": "Shr1_Radeshyam_Khare_Another_vs_The_State_Of_Madhya_Pradesh_Others_on_30_September_1958_1.PDF"}, "year": {"0": 1964, "1": 1954, "2": 1960, "3": 1964, "4": 1958}, "score": {"0": 0.485, "1": 0.48, "2": 0.469, "3": 0.467, "4": 0.466}, "preview": {"0": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "1": "PERSON PERSON PERSON state uttar pradesh union march shyam lal state uttar pradesh union march citations air scr ORG ORG PERSON PERSON PERSON PERSON PERSON state uttar pradesh ORG ORG", "2": "GPE PERSON PERSON another DATE GPE PERSON PERSON another DATE citations air scr air ORG ORG ORG scr scr scr PERSON PERSON PERSON PERSON ORG ORG ORG ORG ORG ORG", "3": "PERSON PERSON PERSON PERSON PERSON andhra pradesh march kanumukkala krishna murthy state andhra pradesh march citations air scr air ORG ORG scwr madljcri scj raghubar dayal raghubar dayal PERSON PERSON", "4": "PERSON PERSON khare another state madhya pradesh others DATE shr radeshyam khare another state madhya pradesh others DATE citations air scr supl air ORG ORG mplj scj scr natwarlal bhagwati"}}</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0.4734</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1954": 1, "1960": 1, "1958": 1}</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>that, rules, commission, state, was</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Mahendra_Bhaskar_Limaye_vs_Union_Of_India_Thr_Secretary_on_20_October_2023.PDF</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:08:44.053987</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "1": "Shyam_Lal_vs_1_The_State_Of_Uttar_Pradesh2_The_Union_on_30_March_1954_1.PDF", "2": "T_Cajee_vs_U_Jormanik_Siem_And_Another_on_20_September_1960_1.PDF", "3": "Kanumukkala_Krishna_Murthy_vs_State_Of_Andhra_Pradesh_on_23_March_1964_1.PDF", "4": "Shr1_Radeshyam_Khare_Another_vs_The_State_Of_Madhya_Pradesh_Others_on_30_September_1958_1.PDF"}, "year": {"0": 1964, "1": 1954, "2": 1960, "3": 1964, "4": 1958}, "score": {"0": 0.485, "1": 0.48, "2": 0.469, "3": 0.467, "4": 0.466}, "preview": {"0": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "1": "PERSON PERSON PERSON state uttar pradesh union march shyam lal state uttar pradesh union march citations air scr ORG ORG PERSON PERSON PERSON PERSON PERSON state uttar pradesh ORG ORG", "2": "GPE PERSON PERSON another DATE GPE PERSON PERSON another DATE citations air scr air ORG ORG ORG scr scr scr PERSON PERSON PERSON PERSON ORG ORG ORG ORG ORG ORG", "3": "PERSON PERSON PERSON PERSON PERSON andhra pradesh march kanumukkala krishna murthy state andhra pradesh march citations air scr air ORG ORG scwr madljcri scj raghubar dayal raghubar dayal PERSON PERSON", "4": "PERSON PERSON khare another state madhya pradesh others DATE shr radeshyam khare another state madhya pradesh others DATE citations air scr supl air ORG ORG mplj scj scr natwarlal bhagwati"}}</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0.4734</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1954": 1, "1960": 1, "1958": 1}</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>that, rules, commission, state, was</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mahendra_Bhaskar_Limaye_vs_Union_Of_India_Thr_Secretary_on_20_October_2023.PDF</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:15:28.060898</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "1": "Shyam_Lal_vs_1_The_State_Of_Uttar_Pradesh2_The_Union_on_30_March_1954_1.PDF", "2": "T_Cajee_vs_U_Jormanik_Siem_And_Another_on_20_September_1960_1.PDF", "3": "Kanumukkala_Krishna_Murthy_vs_State_Of_Andhra_Pradesh_on_23_March_1964_1.PDF", "4": "Shr1_Radeshyam_Khare_Another_vs_The_State_Of_Madhya_Pradesh_Others_on_30_September_1958_1.PDF"}, "year": {"0": 1964, "1": 1954, "2": 1960, "3": 1964, "4": 1958}, "score": {"0": 0.485, "1": 0.48, "2": 0.469, "3": 0.467, "4": 0.466}, "preview": {"0": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "1": "PERSON PERSON PERSON state uttar pradesh union march shyam lal state uttar pradesh union march citations air scr ORG ORG PERSON PERSON PERSON PERSON PERSON state uttar pradesh ORG ORG", "2": "GPE PERSON PERSON another DATE GPE PERSON PERSON another DATE citations air scr air ORG ORG ORG scr scr scr PERSON PERSON PERSON PERSON ORG ORG ORG ORG ORG ORG", "3": "PERSON PERSON PERSON PERSON PERSON andhra pradesh march kanumukkala krishna murthy state andhra pradesh march citations air scr air ORG ORG scwr madljcri scj raghubar dayal raghubar dayal PERSON PERSON", "4": "PERSON PERSON khare another state madhya pradesh others DATE shr radeshyam khare another state madhya pradesh others DATE citations air scr supl air ORG ORG mplj scj scr natwarlal bhagwati"}}</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0.4734</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1954": 1, "1960": 1, "1958": 1}</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>that, rules, commission, state, was</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Mahendra_Bhaskar_Limaye_vs_Union_Of_India_Thr_Secretary_on_20_October_2023.PDF</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:23:00.837742</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "1": "Shyam_Lal_vs_1_The_State_Of_Uttar_Pradesh2_The_Union_on_30_March_1954_1.PDF", "2": "T_Cajee_vs_U_Jormanik_Siem_And_Another_on_20_September_1960_1.PDF", "3": "Kanumukkala_Krishna_Murthy_vs_State_Of_Andhra_Pradesh_on_23_March_1964_1.PDF", "4": "Shr1_Radeshyam_Khare_Another_vs_The_State_Of_Madhya_Pradesh_Others_on_30_September_1958_1.PDF"}, "year": {"0": 1964, "1": 1954, "2": 1960, "3": 1964, "4": 1958}, "score": {"0": 0.485, "1": 0.48, "2": 0.469, "3": 0.467, "4": 0.466}, "preview": {"0": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "1": "PERSON PERSON PERSON state uttar pradesh union march shyam lal state uttar pradesh union march citations air scr ORG ORG PERSON PERSON PERSON PERSON PERSON state uttar pradesh ORG ORG", "2": "GPE PERSON PERSON another DATE GPE PERSON PERSON another DATE citations air scr air ORG ORG ORG scr scr scr PERSON PERSON PERSON PERSON ORG ORG ORG ORG ORG ORG", "3": "PERSON PERSON PERSON PERSON PERSON andhra pradesh march kanumukkala krishna murthy state andhra pradesh march citations air scr air ORG ORG scwr madljcri scj raghubar dayal raghubar dayal PERSON PERSON", "4": "PERSON PERSON khare another state madhya pradesh others DATE shr radeshyam khare another state madhya pradesh others DATE citations air scr supl air ORG ORG mplj scj scr natwarlal bhagwati"}}</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0.4734</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1954": 1, "1960": 1, "1958": 1}</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>that, rules, commission, state, was</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Mahendra_Bhaskar_Limaye_vs_Union_Of_India_Thr_Secretary_on_20_October_2023.PDF</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:36:52.783460</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "1": "Shyam_Lal_vs_1_The_State_Of_Uttar_Pradesh2_The_Union_on_30_March_1954_1.PDF", "2": "T_Cajee_vs_U_Jormanik_Siem_And_Another_on_20_September_1960_1.PDF", "3": "Kanumukkala_Krishna_Murthy_vs_State_Of_Andhra_Pradesh_on_23_March_1964_1.PDF", "4": "Shr1_Radeshyam_Khare_Another_vs_The_State_Of_Madhya_Pradesh_Others_on_30_September_1958_1.PDF"}, "year": {"0": 1964, "1": 1954, "2": 1960, "3": 1964, "4": 1958}, "score": {"0": 0.485, "1": 0.48, "2": 0.469, "3": 0.467, "4": 0.466}, "preview": {"0": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "1": "PERSON PERSON PERSON state uttar pradesh union march shyam lal state uttar pradesh union march citations air scr ORG ORG PERSON PERSON PERSON PERSON PERSON state uttar pradesh ORG ORG", "2": "GPE PERSON PERSON another DATE GPE PERSON PERSON another DATE citations air scr air ORG ORG ORG scr scr scr PERSON PERSON PERSON PERSON ORG ORG ORG ORG ORG ORG", "3": "PERSON PERSON PERSON PERSON PERSON andhra pradesh march kanumukkala krishna murthy state andhra pradesh march citations air scr air ORG ORG scwr madljcri scj raghubar dayal raghubar dayal PERSON PERSON", "4": "PERSON PERSON khare another state madhya pradesh others DATE shr radeshyam khare another state madhya pradesh others DATE citations air scr supl air ORG ORG mplj scj scr natwarlal bhagwati"}}</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0.4734</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1954": 1, "1960": 1, "1958": 1}</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>that, rules, commission, state, was</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sushil_Pandey_vs_The_State_Of_Uttar_Pradesh_Thr_Principal_on_16_January_2023_1.PDF</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:39:12.145788</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF", "1": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "2": "G_S_Ramaswamy_Ors_vs_Inspector_General_Of_Police_Mysore_on_21_January_1964_1.PDF", "3": "The_State_Of_Andhra_vs_Gaddam_Venkatappayya_on_8_December_1960_1.PDF", "4": "The_High_Court_Calcutta_vs_Amal_Kumar_Roy_on_9_April_1962_1.PDF"}, "year": {"0": 1959, "1": 1964, "2": 1964, "3": 1960, "4": 1962}, "score": {"0": 0.73, "1": 0.551, "2": 0.54, "3": 0.538, "4": 0.493}, "preview": {"0": "nagarajan ors state karnataka ors etc may nagarajan ors state karnataka ors etc may citations air scr nagarajan ors state karnataka ors etc date koshal ORG ORG krishnaiyer PERSON PERSON", "1": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "2": "ORG ORG ORG ORG ORG ORG police mysore DATE ramaswamy ors inspectorgeneral police mysore DATE citations air scr air ORG ORG faclr scr PERSON ilr GPE PERSON PERSON ORG ORG", "3": "state andhra PERSON PERSON DATE state andhra PERSON PERSON DATE citations air scr air ORG ORG scj scr scr scr scj scj PERSON PERSON ayyangar ORG ORG ORG ORG ORG", "4": "calcutta amal PERSON PERSON DATE calcutta amal PERSON PERSON DATE citations air scr air ORG ORG bhuvneshwar sinha bhuvneshwar sinha rajagopala ayyangar PERSON PERSON calcutta amal kumar roy date sinha"}}</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0.5704</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1959": 1, "1960": 1, "1962": 1}</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>seniority, that, list, been, direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sushil_Pandey_vs_The_State_Of_Uttar_Pradesh_Thr_Principal_on_16_January_2023_1.PDF</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:41:12.806044</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF", "1": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "2": "G_S_Ramaswamy_Ors_vs_Inspector_General_Of_Police_Mysore_on_21_January_1964_1.PDF", "3": "The_State_Of_Andhra_vs_Gaddam_Venkatappayya_on_8_December_1960_1.PDF", "4": "The_High_Court_Calcutta_vs_Amal_Kumar_Roy_on_9_April_1962_1.PDF"}, "year": {"0": 1959, "1": 1964, "2": 1964, "3": 1960, "4": 1962}, "score": {"0": 0.73, "1": 0.551, "2": 0.54, "3": 0.538, "4": 0.493}, "preview": {"0": "nagarajan ors state karnataka ors etc may nagarajan ors state karnataka ors etc may citations air scr nagarajan ors state karnataka ors etc date koshal ORG ORG krishnaiyer PERSON PERSON", "1": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "2": "ORG ORG ORG ORG ORG ORG police mysore DATE ramaswamy ors inspectorgeneral police mysore DATE citations air scr air ORG ORG faclr scr PERSON ilr GPE PERSON PERSON ORG ORG", "3": "state andhra PERSON PERSON DATE state andhra PERSON PERSON DATE citations air scr air ORG ORG scj scr scr scr scj scj PERSON PERSON ayyangar ORG ORG ORG ORG ORG", "4": "calcutta amal PERSON PERSON DATE calcutta amal PERSON PERSON DATE citations air scr air ORG ORG bhuvneshwar sinha bhuvneshwar sinha rajagopala ayyangar PERSON PERSON calcutta amal kumar roy date sinha"}}</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.5704</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1959": 1, "1960": 1, "1962": 1}</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>seniority, that, list, been, direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Sushil_Pandey_vs_The_State_Of_Uttar_Pradesh_Thr_Principal_on_16_January_2023_1.PDF</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:43:49.073337</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF", "1": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "2": "G_S_Ramaswamy_Ors_vs_Inspector_General_Of_Police_Mysore_on_21_January_1964_1.PDF", "3": "The_State_Of_Andhra_vs_Gaddam_Venkatappayya_on_8_December_1960_1.PDF", "4": "The_High_Court_Calcutta_vs_Amal_Kumar_Roy_on_9_April_1962_1.PDF"}, "year": {"0": 1959, "1": 1964, "2": 1964, "3": 1960, "4": 1962}, "score": {"0": 0.73, "1": 0.551, "2": 0.54, "3": 0.538, "4": 0.493}, "preview": {"0": "nagarajan ors state karnataka ors etc may nagarajan ors state karnataka ors etc may citations air scr nagarajan ors state karnataka ors etc date koshal ORG ORG krishnaiyer PERSON PERSON", "1": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "2": "ORG ORG ORG ORG ORG ORG police mysore DATE ramaswamy ors inspectorgeneral police mysore DATE citations air scr air ORG ORG faclr scr PERSON ilr GPE PERSON PERSON ORG ORG", "3": "state andhra PERSON PERSON DATE state andhra PERSON PERSON DATE citations air scr air ORG ORG scj scr scr scr scj scj PERSON PERSON ayyangar ORG ORG ORG ORG ORG", "4": "calcutta amal PERSON PERSON DATE calcutta amal PERSON PERSON DATE citations air scr air ORG ORG bhuvneshwar sinha bhuvneshwar sinha rajagopala ayyangar PERSON PERSON calcutta amal kumar roy date sinha"}}</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.5704</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1959": 1, "1960": 1, "1962": 1}</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>seniority, that, list, been, direct</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sushil_Pandey_vs_The_State_Of_Uttar_Pradesh_Thr_Principal_on_16_January_2023_1.PDF</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:48:42.906134</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF", "1": "State_Of_Mysore_Anr_vs_K_N_Chandrasekhara_Ors_on_31_July_1964_1.PDF", "2": "G_S_Ramaswamy_Ors_vs_Inspector_General_Of_Police_Mysore_on_21_January_1964_1.PDF", "3": "The_State_Of_Andhra_vs_Gaddam_Venkatappayya_on_8_December_1960_1.PDF", "4": "The_High_Court_Calcutta_vs_Amal_Kumar_Roy_on_9_April_1962_1.PDF"}, "year": {"0": 1959, "1": 1964, "2": 1964, "3": 1960, "4": 1962}, "score": {"0": 0.73, "1": 0.551, "2": 0.54, "3": 0.538, "4": 0.493}, "preview": {"0": "nagarajan ors state karnataka ors etc may nagarajan ors state karnataka ors etc may citations air scr nagarajan ors state karnataka ors etc date koshal ORG ORG krishnaiyer PERSON PERSON", "1": "state mysore anr ORG ORG ors DATE state mysore anr ORG ORG ors DATE ORG ORG ORG ORG PERSON PERSON PERSON PERSON dayal state mysore anr ORG ORG ORG ORG", "2": "ORG ORG ORG ORG ORG ORG police mysore DATE ramaswamy ors inspectorgeneral police mysore DATE citations air scr air ORG ORG faclr scr PERSON ilr GPE PERSON PERSON ORG ORG", "3": "state andhra PERSON PERSON DATE state andhra PERSON PERSON DATE citations air scr air ORG ORG scj scr scr scr scj scj PERSON PERSON ayyangar ORG ORG ORG ORG ORG", "4": "calcutta amal PERSON PERSON DATE calcutta amal PERSON PERSON DATE citations air scr air ORG ORG bhuvneshwar sinha bhuvneshwar sinha rajagopala ayyangar PERSON PERSON calcutta amal kumar roy date sinha"}}</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.5704</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>B_N_Nagarajan_And_Ors_vs_State_Of_Karnataka_And_Ors_Etc_on_3_May_1959_1.PDF</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>{"1964": 2, "1959": 1, "1960": 1, "1962": 1}</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>&lt;Compressed Sparse Row sparse matrix of dtype 'float64'
+	with 1603441 stored elements and shape (3126, 5000)&gt;
+  Coords	Values
+  (0, 3135)	0.08442848526897538
+  (0, 2127)	0.06268903758533283
+  (0, 156)	0.03580765847167488
+  (0, 2455)	0.09044280818340414
+  (0, 4047)	0.016901516133891348
+  (0, 3679)	0.010146287077737414
+  (0, 770)	0.00572349894504952
+  (0, 4301)	0.07448044260301412
+  (0, 4875)	0.07536900681950345
+  (0, 870)	0.3818011374134117
+  (0, 1550)	0.06000628641846781
+  (0, 1442)	0.010088789804717425
+  (0, 2716)	0.056000948839333126
+  (0, 127)	0.054427985040539445
+  (0, 3836)	0.013618904456853284
+  (0, 1409)	0.11412736468605973
+  (0, 458)	0.012789168271996722
+  (0, 2003)	0.021487528182783756
+  (0, 2806)	0.04032262614928743
+  (0, 316)	0.04564632880884472
+  (0, 2956)	0.021074952288090365
+  (0, 3978)	0.13747389084659417
+  (0, 4193)	0.3499060347540356
+  (0, 2754)	0.020835716065565734
+  (0, 4858)	0.04971084683499533
+  :	:
+  (3125, 3286)	0.008479767375246467
+  (3125, 261)	0.007406066466346979
+  (3125, 2531)	0.004882273932699915
+  (3125, 830)	0.009180521667769889
+  (3125, 1246)	0.015617363828688474
+  (3125, 4340)	0.007103951285935974
+  (3125, 4246)	0.018682314978079588
+  (3125, 2805)	0.009239334550479684
+  (3125, 2749)	0.009013333379401368
+  (3125, 4784)	0.008438580562274584
+  (3125, 744)	0.018809399471310696
+  (3125, 3356)	0.05376256228764081
+  (3125, 3705)	0.009219547317313058
+  (3125, 1387)	0.5267120961993962
+  (3125, 3805)	0.02406195569455651
+  (3125, 4621)	0.01847866910095937
+  (3125, 3417)	0.016270417250408578
+  (3125, 4075)	0.004779217725009713
+  (3125, 1125)	0.05103031198068071
+  (3125, 1206)	0.007944013457917848
+  (3125, 1126)	0.010335784873717412
+  (3125, 1132)	0.009104573814055746
+  (3125, 953)	0.10881122705239876
+  (3125, 4063)	0.009754783018765664
+  (3125, 2670)	0.007758861039575557</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analytics functions to use subset embeddings for keyword search results and improve word cloud generation
</commit_message>
<xml_diff>
--- a/data/history.xlsx
+++ b/data/history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,6 +495,41 @@
         </is>
       </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>{"file_name": {"0": "The_State_Of_Uttar_Pradesh_vs_Bhagwant_Kishore_Joshi_on_17_April_1963_1.PDF", "1": "H_N_Rishbud_And_Inder_Singh_vs_The_State_Of_Delhi_And_Connected_on_14_December_1954_1.PDF", "2": "Purshottam_Jethanand_vs_The_State_Of_Kutch_on_5_March_1954_1.PDF", "3": "Macherla_Hanumantha_Raoand_Others_vs_The_State_Of_Andhra_Pradesh_With_on_17_September_1957_1.PDF", "4": "Niranjan_Singh_vs_The_State_Of_Uttar_Pradesh_And_on_3_October_1956_1.PDF"}, "year": {"0": 1963, "1": 1954, "2": 1954, "3": 1957, "4": 1956}, "score": {"0": 0.621, "1": 0.613, "2": 0.574, "3": 0.546, "4": 0.544}, "preview": {"0": "state uttar pradesh bhagwant PERSON PERSON DATE state uttar pradesh bhagwant PERSON PERSON DATE citations air scr air ORG ORG lablj PERSON scd scr ilr raghubar dayal PERSON PERSON state", "1": "rishbud inder GPE state delhiand connected DATE rishbud inder GPE state delhiand connected DATE citations air scr air ORG ORG pun PERSON PERSON jagannadhadas PERSON PERSON bose rishbud inder singh", "2": "PERSON PERSON PERSON state kutch march purshottam jethanand state kutch march citations air jagannadhas special leave appellant police jamadar working local investigation branch mandvi state kutch prosecution visited place called", "3": "PERSON PERSON raoand others state andhra pradeshwith DATE macherla hanumantha raoand others state andhra pradeshwith DATE citations air scr air ORG ORG bljr PERSON PERSON scj bhuvneshwar sinha bhuvneshwar sinha", "4": "PERSON PERSON state uttar pradeshand DATE niranjan ORG state uttar pradeshand DATE citations air scr air ORG ORG madljcri ilr govinda menon ORG ORG natwarlal ORG ORG ORG ORG ORG"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Y_Balaji_vs_Karthik_Desari_on_16_May_2023_1.PDF</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-03 13:19:34.174773</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5796</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The_State_Of_Uttar_Pradesh_vs_Bhagwant_Kishore_Joshi_on_17_April_1963_1.PDF</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>that, was, high, not, order</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>{"1954": 2, "1963": 1, "1957": 1, "1956": 1}</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>{"file_name": {"0": "The_State_Of_Uttar_Pradesh_vs_Bhagwant_Kishore_Joshi_on_17_April_1963_1.PDF", "1": "H_N_Rishbud_And_Inder_Singh_vs_The_State_Of_Delhi_And_Connected_on_14_December_1954_1.PDF", "2": "Purshottam_Jethanand_vs_The_State_Of_Kutch_on_5_March_1954_1.PDF", "3": "Macherla_Hanumantha_Raoand_Others_vs_The_State_Of_Andhra_Pradesh_With_on_17_September_1957_1.PDF", "4": "Niranjan_Singh_vs_The_State_Of_Uttar_Pradesh_And_on_3_October_1956_1.PDF"}, "year": {"0": 1963, "1": 1954, "2": 1954, "3": 1957, "4": 1956}, "score": {"0": 0.621, "1": 0.613, "2": 0.574, "3": 0.546, "4": 0.544}, "preview": {"0": "state uttar pradesh bhagwant PERSON PERSON DATE state uttar pradesh bhagwant PERSON PERSON DATE citations air scr air ORG ORG lablj PERSON scd scr ilr raghubar dayal PERSON PERSON state", "1": "rishbud inder GPE state delhiand connected DATE rishbud inder GPE state delhiand connected DATE citations air scr air ORG ORG pun PERSON PERSON jagannadhadas PERSON PERSON bose rishbud inder singh", "2": "PERSON PERSON PERSON state kutch march purshottam jethanand state kutch march citations air jagannadhas special leave appellant police jamadar working local investigation branch mandvi state kutch prosecution visited place called", "3": "PERSON PERSON raoand others state andhra pradeshwith DATE macherla hanumantha raoand others state andhra pradeshwith DATE citations air scr air ORG ORG bljr PERSON PERSON scj bhuvneshwar sinha bhuvneshwar sinha", "4": "PERSON PERSON state uttar pradeshand DATE niranjan ORG state uttar pradeshand DATE citations air scr air ORG ORG madljcri ilr govinda menon ORG ORG natwarlal ORG ORG ORG ORG ORG"}}</t>
         </is>

</xml_diff>